<commit_message>
OS LR 1 solution, report, IAD PR solution fixes
</commit_message>
<xml_diff>
--- a/BSUIR/semestre 5/IAD/ИАД ПР.xlsx
+++ b/BSUIR/semestre 5/IAD/ИАД ПР.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="23001"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="22527"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Goodvin\Documents\GitHub\study-repos\BSUIR\semestre 5\IAD\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\minsk\Documents\GitHub\study-repos\BSUIR\semestre 5\IAD\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{75FB3E5A-FC2D-4D80-9C15-981D0F907239}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{454B0233-15FA-405C-B97E-49E1272B5AEE}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="12000" yWindow="945" windowWidth="14880" windowHeight="18450" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="5115" yWindow="1035" windowWidth="15375" windowHeight="7875" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Задание 1" sheetId="1" r:id="rId1"/>
@@ -15701,7 +15701,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{86F3EFB3-6972-4806-8863-49B25B9B0C7C}">
-  <dimension ref="A1:E21"/>
+  <dimension ref="A1:E28"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="4" max="4" width="13.5703125" customWidth="1"/>
@@ -15810,6 +15810,10 @@
       <c r="D9" s="8" t="s">
         <v>33</v>
       </c>
+      <c r="E9">
+        <f>_xlfn.NORM.DIST(A2,$E$2,1,TRUE)</f>
+        <v>7.1428107352713589E-3</v>
+      </c>
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A10">
@@ -15818,6 +15822,10 @@
       <c r="B10">
         <v>200</v>
       </c>
+      <c r="E10">
+        <f t="shared" ref="E10:E37" si="0">_xlfn.NORM.DIST(A3,$E$2,1,TRUE)</f>
+        <v>0.99461385404593328</v>
+      </c>
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A11">
@@ -15826,6 +15834,10 @@
       <c r="B11">
         <v>130</v>
       </c>
+      <c r="E11">
+        <f t="shared" si="0"/>
+        <v>2.8029327681617391E-4</v>
+      </c>
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A12">
@@ -15834,6 +15846,10 @@
       <c r="B12">
         <v>140</v>
       </c>
+      <c r="E12">
+        <f t="shared" si="0"/>
+        <v>7.3529259609647943E-2</v>
+      </c>
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A13">
@@ -15842,6 +15858,10 @@
       <c r="B13">
         <v>265</v>
       </c>
+      <c r="E13">
+        <f t="shared" si="0"/>
+        <v>0.70884031321165264</v>
+      </c>
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A14">
@@ -15850,6 +15870,10 @@
       <c r="B14">
         <v>185</v>
       </c>
+      <c r="E14">
+        <f t="shared" si="0"/>
+        <v>4.2935144699718097E-6</v>
+      </c>
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A15">
@@ -15858,6 +15882,10 @@
       <c r="B15">
         <v>112</v>
       </c>
+      <c r="E15">
+        <f t="shared" si="0"/>
+        <v>2.5184910054460716E-8</v>
+      </c>
     </row>
     <row r="16" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A16">
@@ -15866,45 +15894,111 @@
       <c r="B16">
         <v>140</v>
       </c>
-    </row>
-    <row r="17" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="E16">
+        <f t="shared" si="0"/>
+        <v>7.3529259609647943E-2</v>
+      </c>
+    </row>
+    <row r="17" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A17">
         <v>71</v>
       </c>
       <c r="B17">
         <v>150</v>
       </c>
-    </row>
-    <row r="18" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="E17">
+        <f t="shared" si="0"/>
+        <v>0.9999973177042204</v>
+      </c>
+    </row>
+    <row r="18" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A18">
         <v>74</v>
       </c>
       <c r="B18">
         <v>165</v>
       </c>
-    </row>
-    <row r="19" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="E18">
+        <f t="shared" si="0"/>
+        <v>2.8029327681617391E-4</v>
+      </c>
+    </row>
+    <row r="19" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A19">
         <v>75</v>
       </c>
       <c r="B19">
         <v>185</v>
       </c>
-    </row>
-    <row r="20" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="E19">
+        <f t="shared" si="0"/>
+        <v>0.70884031321165264</v>
+      </c>
+    </row>
+    <row r="20" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A20">
         <v>75</v>
       </c>
       <c r="B20">
         <v>210</v>
       </c>
-    </row>
-    <row r="21" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="E20">
+        <f t="shared" si="0"/>
+        <v>0.99999999999997824</v>
+      </c>
+    </row>
+    <row r="21" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A21">
         <v>76</v>
       </c>
       <c r="B21">
         <v>220</v>
+      </c>
+      <c r="E21">
+        <f t="shared" si="0"/>
+        <v>0.99461385404593328</v>
+      </c>
+    </row>
+    <row r="22" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="E22">
+        <f t="shared" si="0"/>
+        <v>4.2935144699718097E-6</v>
+      </c>
+    </row>
+    <row r="23" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="E23">
+        <f t="shared" si="0"/>
+        <v>2.5184910054460716E-8</v>
+      </c>
+    </row>
+    <row r="24" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="E24">
+        <f>_xlfn.NORM.DIST(A17,$E$2,1,TRUE)</f>
+        <v>0.32635522028791897</v>
+      </c>
+    </row>
+    <row r="25" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="E25">
+        <f t="shared" si="0"/>
+        <v>0.99461385404593328</v>
+      </c>
+    </row>
+    <row r="26" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="E26">
+        <f>_xlfn.NORM.DIST(A19,$E$2,1,TRUE)</f>
+        <v>0.99980738442436434</v>
+      </c>
+    </row>
+    <row r="27" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="E27">
+        <f>_xlfn.NORM.DIST(A20,$E$2,1,TRUE)</f>
+        <v>0.99980738442436434</v>
+      </c>
+    </row>
+    <row r="28" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="E28">
+        <f>_xlfn.NORM.DIST(A21,$E$2,1,TRUE)</f>
+        <v>0.9999973177042204</v>
       </c>
     </row>
   </sheetData>

</xml_diff>